<commit_message>
FarmacogeneticReport.py now works on the template. HLA-B*1502 was added back in.
</commit_message>
<xml_diff>
--- a/Output/Diagnostics/unknowns.xlsx
+++ b/Output/Diagnostics/unknowns.xlsx
@@ -660,7 +660,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
@@ -677,7 +677,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
@@ -694,7 +694,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -711,7 +711,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
@@ -728,7 +728,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -745,7 +745,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -762,7 +762,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -779,7 +779,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -796,7 +796,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B13" t="s">
         <v>8</v>
@@ -813,7 +813,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B14" t="s">
         <v>8</v>
@@ -830,7 +830,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -844,7 +844,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="B16" t="s">
         <v>9</v>
@@ -858,7 +858,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="B17" t="s">
         <v>10</v>
@@ -875,7 +875,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1">
-        <v>621</v>
+        <v>630</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
@@ -892,7 +892,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
@@ -909,7 +909,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1">
-        <v>915</v>
+        <v>928</v>
       </c>
       <c r="B20" t="s">
         <v>13</v>
@@ -926,7 +926,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1">
-        <v>954</v>
+        <v>968</v>
       </c>
       <c r="B21" t="s">
         <v>13</v>
@@ -940,7 +940,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1">
-        <v>982</v>
+        <v>996</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -954,7 +954,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1">
-        <v>992</v>
+        <v>1006</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -971,7 +971,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1">
-        <v>1056</v>
+        <v>1071</v>
       </c>
       <c r="B24" t="s">
         <v>15</v>
@@ -985,7 +985,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1">
-        <v>1199</v>
+        <v>1216</v>
       </c>
       <c r="B25" t="s">
         <v>16</v>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1">
-        <v>1200</v>
+        <v>1217</v>
       </c>
       <c r="B26" t="s">
         <v>16</v>
@@ -1019,7 +1019,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1">
-        <v>1238</v>
+        <v>1256</v>
       </c>
       <c r="B27" t="s">
         <v>16</v>
@@ -1036,7 +1036,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1">
-        <v>1337</v>
+        <v>1356</v>
       </c>
       <c r="B28" t="s">
         <v>17</v>
@@ -1053,7 +1053,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1">
-        <v>1406</v>
+        <v>1426</v>
       </c>
       <c r="B29" t="s">
         <v>18</v>
@@ -1070,7 +1070,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1">
-        <v>1407</v>
+        <v>1427</v>
       </c>
       <c r="B30" t="s">
         <v>18</v>
@@ -1087,7 +1087,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1">
-        <v>1599</v>
+        <v>1622</v>
       </c>
       <c r="B31" t="s">
         <v>19</v>
@@ -1104,7 +1104,7 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1">
-        <v>1613</v>
+        <v>1636</v>
       </c>
       <c r="B32" t="s">
         <v>19</v>
@@ -1121,7 +1121,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="1">
-        <v>1615</v>
+        <v>1638</v>
       </c>
       <c r="B33" t="s">
         <v>19</v>
@@ -1138,7 +1138,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="1">
-        <v>1672</v>
+        <v>1696</v>
       </c>
       <c r="B34" t="s">
         <v>20</v>
@@ -1152,7 +1152,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="1">
-        <v>1744</v>
+        <v>1769</v>
       </c>
       <c r="B35" t="s">
         <v>21</v>
@@ -1169,7 +1169,7 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="1">
-        <v>1806</v>
+        <v>1832</v>
       </c>
       <c r="B36" t="s">
         <v>22</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="1">
-        <v>1810</v>
+        <v>1836</v>
       </c>
       <c r="B37" t="s">
         <v>22</v>
@@ -1200,7 +1200,7 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="1">
-        <v>1815</v>
+        <v>1841</v>
       </c>
       <c r="B38" t="s">
         <v>22</v>
@@ -1214,7 +1214,7 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1">
-        <v>1826</v>
+        <v>1852</v>
       </c>
       <c r="B39" t="s">
         <v>22</v>
@@ -1228,7 +1228,7 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="1">
-        <v>1838</v>
+        <v>1865</v>
       </c>
       <c r="B40" t="s">
         <v>22</v>
@@ -1245,7 +1245,7 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1">
-        <v>1839</v>
+        <v>1866</v>
       </c>
       <c r="B41" t="s">
         <v>22</v>
@@ -1262,7 +1262,7 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="1">
-        <v>1851</v>
+        <v>1878</v>
       </c>
       <c r="B42" t="s">
         <v>22</v>
@@ -1276,7 +1276,7 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="1">
-        <v>1958</v>
+        <v>1986</v>
       </c>
       <c r="B43" t="s">
         <v>23</v>
@@ -1293,7 +1293,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="1">
-        <v>2224</v>
+        <v>2256</v>
       </c>
       <c r="B44" t="s">
         <v>24</v>
@@ -1307,7 +1307,7 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="1">
-        <v>2240</v>
+        <v>2272</v>
       </c>
       <c r="B45" t="s">
         <v>24</v>
@@ -1321,7 +1321,7 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="1">
-        <v>2253</v>
+        <v>2286</v>
       </c>
       <c r="B46" t="s">
         <v>24</v>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="1">
-        <v>2265</v>
+        <v>2298</v>
       </c>
       <c r="B47" t="s">
         <v>24</v>
@@ -1352,7 +1352,7 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="1">
-        <v>2277</v>
+        <v>2310</v>
       </c>
       <c r="B48" t="s">
         <v>25</v>
@@ -1369,7 +1369,7 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="1">
-        <v>2346</v>
+        <v>2380</v>
       </c>
       <c r="B49" t="s">
         <v>26</v>
@@ -1386,7 +1386,7 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="1">
-        <v>2354</v>
+        <v>2388</v>
       </c>
       <c r="B50" t="s">
         <v>26</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="1">
-        <v>2372</v>
+        <v>2406</v>
       </c>
       <c r="B51" t="s">
         <v>26</v>
@@ -1420,7 +1420,7 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="1">
-        <v>2708</v>
+        <v>2747</v>
       </c>
       <c r="B52" t="s">
         <v>27</v>
@@ -1437,7 +1437,7 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="1">
-        <v>2712</v>
+        <v>2751</v>
       </c>
       <c r="B53" t="s">
         <v>27</v>
@@ -1451,7 +1451,7 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="1">
-        <v>2717</v>
+        <v>2756</v>
       </c>
       <c r="B54" t="s">
         <v>27</v>
@@ -1468,7 +1468,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="1">
-        <v>3219</v>
+        <v>3266</v>
       </c>
       <c r="B55" t="s">
         <v>28</v>
@@ -1485,7 +1485,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="1">
-        <v>3237</v>
+        <v>3284</v>
       </c>
       <c r="B56" t="s">
         <v>28</v>
@@ -1502,7 +1502,7 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="1">
-        <v>3333</v>
+        <v>3381</v>
       </c>
       <c r="B57" t="s">
         <v>29</v>
@@ -1516,7 +1516,7 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="1">
-        <v>3334</v>
+        <v>3382</v>
       </c>
       <c r="B58" t="s">
         <v>29</v>
@@ -1533,7 +1533,7 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="1">
-        <v>3344</v>
+        <v>3392</v>
       </c>
       <c r="B59" t="s">
         <v>29</v>
@@ -1547,7 +1547,7 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="1">
-        <v>3407</v>
+        <v>3456</v>
       </c>
       <c r="B60" t="s">
         <v>30</v>
@@ -1564,7 +1564,7 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="1">
-        <v>3614</v>
+        <v>3666</v>
       </c>
       <c r="B61" t="s">
         <v>31</v>
@@ -1581,7 +1581,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="1">
-        <v>3738</v>
+        <v>3792</v>
       </c>
       <c r="B62" t="s">
         <v>32</v>
@@ -1598,7 +1598,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="1">
-        <v>3890</v>
+        <v>3946</v>
       </c>
       <c r="B63" t="s">
         <v>33</v>
@@ -1615,7 +1615,7 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="1">
-        <v>4023</v>
+        <v>4081</v>
       </c>
       <c r="B64" t="s">
         <v>34</v>
@@ -1632,7 +1632,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="1">
-        <v>4071</v>
+        <v>4130</v>
       </c>
       <c r="B65" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
Alles werkt, behalve diagnostics
</commit_message>
<xml_diff>
--- a/Output/Diagnostics/unknowns.xlsx
+++ b/Output/Diagnostics/unknowns.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="99">
   <si>
     <t>sample_id</t>
   </si>
@@ -28,211 +28,289 @@
     <t>genotype</t>
   </si>
   <si>
-    <t>BFX0034312</t>
-  </si>
-  <si>
-    <t>BFX0034487</t>
-  </si>
-  <si>
-    <t>D402007253</t>
-  </si>
-  <si>
-    <t>D402007309</t>
-  </si>
-  <si>
-    <t>G001040505</t>
-  </si>
-  <si>
-    <t>G001040523</t>
-  </si>
-  <si>
-    <t>G001040547</t>
-  </si>
-  <si>
-    <t>G001040552</t>
-  </si>
-  <si>
-    <t>G001040553</t>
-  </si>
-  <si>
-    <t>G001040582</t>
-  </si>
-  <si>
-    <t>G001040585</t>
-  </si>
-  <si>
-    <t>G001040590</t>
-  </si>
-  <si>
-    <t>G001040596</t>
-  </si>
-  <si>
-    <t>G001040603</t>
-  </si>
-  <si>
-    <t>G001040604</t>
-  </si>
-  <si>
-    <t>G001040609</t>
-  </si>
-  <si>
-    <t>G001040611</t>
-  </si>
-  <si>
-    <t>G001040613</t>
-  </si>
-  <si>
-    <t>G001040615</t>
-  </si>
-  <si>
-    <t>G001040626</t>
-  </si>
-  <si>
-    <t>G001040646</t>
-  </si>
-  <si>
-    <t>G001040649</t>
-  </si>
-  <si>
-    <t>G001040651</t>
-  </si>
-  <si>
-    <t>G001040659</t>
-  </si>
-  <si>
-    <t>G001040672</t>
-  </si>
-  <si>
-    <t>G001040675</t>
-  </si>
-  <si>
-    <t>G001040677</t>
-  </si>
-  <si>
-    <t>G001040681</t>
-  </si>
-  <si>
-    <t>G001040685</t>
-  </si>
-  <si>
-    <t>G001040687</t>
-  </si>
-  <si>
-    <t>G001040694</t>
-  </si>
-  <si>
-    <t>G001040700</t>
-  </si>
-  <si>
-    <t>COMT</t>
-  </si>
-  <si>
-    <t>CYP4F2</t>
-  </si>
-  <si>
-    <t>DPYD</t>
-  </si>
-  <si>
-    <t>CYP2B6</t>
+    <t>G001040554</t>
+  </si>
+  <si>
+    <t>G001040558</t>
+  </si>
+  <si>
+    <t>G001040559</t>
+  </si>
+  <si>
+    <t>G001040560</t>
+  </si>
+  <si>
+    <t>G001040562</t>
+  </si>
+  <si>
+    <t>G001040563</t>
+  </si>
+  <si>
+    <t>G001040565</t>
+  </si>
+  <si>
+    <t>G001040567</t>
+  </si>
+  <si>
+    <t>G001040568</t>
+  </si>
+  <si>
+    <t>G001040569</t>
+  </si>
+  <si>
+    <t>G001040571</t>
+  </si>
+  <si>
+    <t>G001040572</t>
+  </si>
+  <si>
+    <t>G001040573</t>
+  </si>
+  <si>
+    <t>G001040574</t>
+  </si>
+  <si>
+    <t>G001040575</t>
+  </si>
+  <si>
+    <t>G001040576</t>
+  </si>
+  <si>
+    <t>G001040579</t>
+  </si>
+  <si>
+    <t>G001040580</t>
+  </si>
+  <si>
+    <t>G001040583</t>
+  </si>
+  <si>
+    <t>G001040584</t>
+  </si>
+  <si>
+    <t>G001040588</t>
+  </si>
+  <si>
+    <t>G001040598</t>
+  </si>
+  <si>
+    <t>G001040599</t>
+  </si>
+  <si>
+    <t>G001040600</t>
+  </si>
+  <si>
+    <t>G001040653</t>
+  </si>
+  <si>
+    <t>G001040656</t>
+  </si>
+  <si>
+    <t>G001040664</t>
+  </si>
+  <si>
+    <t>G001040671</t>
+  </si>
+  <si>
+    <t>G001040678</t>
+  </si>
+  <si>
+    <t>G001040682</t>
+  </si>
+  <si>
+    <t>G001040683</t>
+  </si>
+  <si>
+    <t>G001040691</t>
+  </si>
+  <si>
+    <t>G001040692</t>
+  </si>
+  <si>
+    <t>G001040695</t>
+  </si>
+  <si>
+    <t>G001040698</t>
+  </si>
+  <si>
+    <t>G001121701</t>
+  </si>
+  <si>
+    <t>G001121702</t>
+  </si>
+  <si>
+    <t>G001121705</t>
+  </si>
+  <si>
+    <t>G001121707</t>
+  </si>
+  <si>
+    <t>G001121708</t>
+  </si>
+  <si>
+    <t>G001121712</t>
+  </si>
+  <si>
+    <t>G001121715</t>
+  </si>
+  <si>
+    <t>G001121717</t>
+  </si>
+  <si>
+    <t>G001121718</t>
+  </si>
+  <si>
+    <t>G001121726</t>
+  </si>
+  <si>
+    <t>G001121729</t>
+  </si>
+  <si>
+    <t>G001121730</t>
+  </si>
+  <si>
+    <t>G001121737</t>
+  </si>
+  <si>
+    <t>G001121740</t>
+  </si>
+  <si>
+    <t>G001121742</t>
+  </si>
+  <si>
+    <t>G001121743</t>
+  </si>
+  <si>
+    <t>G001121745</t>
+  </si>
+  <si>
+    <t>G001121752</t>
+  </si>
+  <si>
+    <t>G001121753</t>
+  </si>
+  <si>
+    <t>G001121757</t>
+  </si>
+  <si>
+    <t>G001121758</t>
+  </si>
+  <si>
+    <t>G001121760</t>
+  </si>
+  <si>
+    <t>G001121763</t>
+  </si>
+  <si>
+    <t>G001121764</t>
+  </si>
+  <si>
+    <t>G001121766</t>
+  </si>
+  <si>
+    <t>G001121768</t>
+  </si>
+  <si>
+    <t>G001121771</t>
+  </si>
+  <si>
+    <t>G001121772</t>
+  </si>
+  <si>
+    <t>G001121773</t>
+  </si>
+  <si>
+    <t>G001121775</t>
+  </si>
+  <si>
+    <t>G001121776</t>
+  </si>
+  <si>
+    <t>G001121777</t>
+  </si>
+  <si>
+    <t>G001121778</t>
+  </si>
+  <si>
+    <t>G001121779</t>
+  </si>
+  <si>
+    <t>G001121780</t>
+  </si>
+  <si>
+    <t>G001121782</t>
+  </si>
+  <si>
+    <t>G001121783</t>
+  </si>
+  <si>
+    <t>G001121784</t>
+  </si>
+  <si>
+    <t>G001121785</t>
+  </si>
+  <si>
+    <t>G001121787</t>
+  </si>
+  <si>
+    <t>G001121788</t>
+  </si>
+  <si>
+    <t>G001121791</t>
+  </si>
+  <si>
+    <t>G001121792</t>
+  </si>
+  <si>
+    <t>G001121793</t>
+  </si>
+  <si>
+    <t>G001121794</t>
+  </si>
+  <si>
+    <t>G001121795</t>
+  </si>
+  <si>
+    <t>G001121796</t>
+  </si>
+  <si>
+    <t>G001121797</t>
+  </si>
+  <si>
+    <t>G001121798</t>
+  </si>
+  <si>
+    <t>G001121799</t>
+  </si>
+  <si>
+    <t>G001121800</t>
+  </si>
+  <si>
+    <t>ABCG2</t>
+  </si>
+  <si>
+    <t>NQ01</t>
   </si>
   <si>
     <t>BChE</t>
   </si>
   <si>
-    <t>BDNF-AS; BDNF</t>
-  </si>
-  <si>
-    <t>CYP2D6</t>
-  </si>
-  <si>
-    <t>Sult1A1</t>
-  </si>
-  <si>
-    <t>RYR1</t>
-  </si>
-  <si>
-    <t>ABCB1</t>
-  </si>
-  <si>
-    <t>CYP2C8</t>
-  </si>
-  <si>
-    <t>CYP2A6</t>
-  </si>
-  <si>
-    <t>UCP2</t>
-  </si>
-  <si>
-    <t>DRD2</t>
-  </si>
-  <si>
-    <t>CYP2C9</t>
-  </si>
-  <si>
-    <t>G6PD</t>
-  </si>
-  <si>
-    <t>MTHFR 1298A&gt;C</t>
-  </si>
-  <si>
-    <t>MTHFR677</t>
-  </si>
-  <si>
-    <t>TNFa</t>
-  </si>
-  <si>
-    <t>CYP2E1</t>
-  </si>
-  <si>
     <t>ERROR</t>
   </si>
   <si>
-    <t>unknown</t>
-  </si>
-  <si>
-    <t>Not_PM</t>
-  </si>
-  <si>
     <t>Not_Determined</t>
   </si>
   <si>
-    <t>*4/*6</t>
-  </si>
-  <si>
-    <t>*1/*15</t>
-  </si>
-  <si>
-    <t>*3/*5</t>
-  </si>
-  <si>
-    <t>*1/*5</t>
+    <t>T/G</t>
+  </si>
+  <si>
+    <t>G/G</t>
+  </si>
+  <si>
+    <t>T/T</t>
   </si>
   <si>
     <t>---</t>
-  </si>
-  <si>
-    <t>*1/*28</t>
-  </si>
-  <si>
-    <t>*1/*11</t>
-  </si>
-  <si>
-    <t>*1/*6</t>
-  </si>
-  <si>
-    <t>*1C/*4+1C</t>
-  </si>
-  <si>
-    <t>*3/*6</t>
-  </si>
-  <si>
-    <t>*1/*2+36</t>
-  </si>
-  <si>
-    <t>*4/*5</t>
-  </si>
-  <si>
-    <t>*7B/*7C</t>
   </si>
 </sst>
 </file>
@@ -590,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -609,1042 +687,1498 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1">
-        <v>27</v>
+        <v>141</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1">
-        <v>87</v>
+        <v>211</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1">
-        <v>96</v>
+        <v>281</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1">
-        <v>166</v>
+        <v>351</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1">
-        <v>218</v>
+        <v>421</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1">
-        <v>219</v>
+        <v>491</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1">
-        <v>222</v>
+        <v>561</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1">
-        <v>236</v>
+        <v>631</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1">
-        <v>288</v>
+        <v>701</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1">
-        <v>301</v>
+        <v>771</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1">
-        <v>340</v>
+        <v>841</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1">
-        <v>371</v>
+        <v>911</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E15" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1">
-        <v>408</v>
+        <v>981</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E16" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1">
-        <v>437</v>
+        <v>1051</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1">
-        <v>630</v>
+        <v>1121</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E18" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1">
-        <v>726</v>
+        <v>1191</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1">
-        <v>928</v>
+        <v>1261</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C20" t="s">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="D20" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="E20" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1">
-        <v>968</v>
+        <v>1331</v>
       </c>
       <c r="B21" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="D21" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E21" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1">
-        <v>996</v>
+        <v>1401</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C22" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="D22" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E22" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1">
-        <v>1006</v>
+        <v>1471</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E23" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1">
-        <v>1071</v>
+        <v>1541</v>
       </c>
       <c r="B24" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E24" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1">
-        <v>1216</v>
+        <v>1611</v>
       </c>
       <c r="B25" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C25" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D25" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1">
-        <v>1217</v>
+        <v>1681</v>
       </c>
       <c r="B26" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C26" t="s">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="D26" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E26" t="s">
-        <v>56</v>
+        <v>95</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1">
-        <v>1256</v>
+        <v>1751</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="C27" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1">
-        <v>1356</v>
+        <v>1821</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C28" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E28" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1">
-        <v>1426</v>
+        <v>1891</v>
       </c>
       <c r="B29" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C29" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D29" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="E29" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1">
-        <v>1427</v>
+        <v>1961</v>
       </c>
       <c r="B30" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C30" t="s">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="D30" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E30" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1">
-        <v>1622</v>
+        <v>2031</v>
       </c>
       <c r="B31" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C31" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="D31" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E31" t="s">
-        <v>56</v>
+        <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1">
-        <v>1636</v>
+        <v>2101</v>
       </c>
       <c r="B32" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="C32" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D32" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E32" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="1">
-        <v>1638</v>
+        <v>2171</v>
       </c>
       <c r="B33" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C33" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
       <c r="D33" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E33" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="1">
-        <v>1696</v>
+        <v>2241</v>
       </c>
       <c r="B34" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C34" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E34" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="1">
-        <v>1769</v>
+        <v>2311</v>
       </c>
       <c r="B35" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C35" t="s">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="D35" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E35" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="1">
-        <v>1832</v>
+        <v>2381</v>
       </c>
       <c r="B36" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C36" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="D36" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E36" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="1">
-        <v>1836</v>
+        <v>2451</v>
       </c>
       <c r="B37" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="D37" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E37" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="1">
-        <v>1841</v>
+        <v>2521</v>
       </c>
       <c r="B38" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="C38" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D38" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E38" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1">
-        <v>1852</v>
+        <v>2591</v>
       </c>
       <c r="B39" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="C39" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="D39" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E39" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="1">
-        <v>1865</v>
+        <v>2661</v>
       </c>
       <c r="B40" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>52</v>
+        <v>90</v>
       </c>
       <c r="D40" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E40" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1">
-        <v>1866</v>
+        <v>2731</v>
       </c>
       <c r="B41" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D41" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E41" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="1">
-        <v>1878</v>
+        <v>2801</v>
       </c>
       <c r="B42" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="C42" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="D42" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E42" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="1">
-        <v>1986</v>
+        <v>2871</v>
       </c>
       <c r="B43" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C43" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D43" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="E43" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="1">
-        <v>2256</v>
+        <v>2941</v>
       </c>
       <c r="B44" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="C44" t="s">
-        <v>47</v>
+        <v>90</v>
       </c>
       <c r="D44" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E44" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="1">
-        <v>2272</v>
+        <v>3011</v>
       </c>
       <c r="B45" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="C45" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="D45" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E45" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="1">
-        <v>2286</v>
+        <v>3081</v>
       </c>
       <c r="B46" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="C46" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D46" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E46" t="s">
-        <v>56</v>
+        <v>95</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="1">
-        <v>2298</v>
+        <v>3151</v>
       </c>
       <c r="B47" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="C47" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="D47" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E47" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="1">
-        <v>2310</v>
+        <v>3221</v>
       </c>
       <c r="B48" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C48" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="D48" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E48" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="1">
-        <v>2380</v>
+        <v>3291</v>
       </c>
       <c r="B49" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="C49" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="D49" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E49" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="1">
-        <v>2388</v>
+        <v>3361</v>
       </c>
       <c r="B50" t="s">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="C50" t="s">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="D50" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
       <c r="E50" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="1">
-        <v>2406</v>
+        <v>3431</v>
       </c>
       <c r="B51" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="C51" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D51" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E51" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="1">
-        <v>2747</v>
+        <v>3501</v>
       </c>
       <c r="B52" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="C52" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="D52" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E52" t="s">
-        <v>61</v>
+        <v>96</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="1">
-        <v>2751</v>
+        <v>3571</v>
       </c>
       <c r="B53" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C53" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D53" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E53" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="1">
-        <v>2756</v>
+        <v>3641</v>
       </c>
       <c r="B54" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="C54" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D54" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E54" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="1">
-        <v>3266</v>
+        <v>3711</v>
       </c>
       <c r="B55" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="C55" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="D55" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E55" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="1">
-        <v>3284</v>
+        <v>3764</v>
       </c>
       <c r="B56" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="C56" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="D56" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
       <c r="E56" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="1">
-        <v>3381</v>
+        <v>3781</v>
       </c>
       <c r="B57" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="C57" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D57" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E57" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="1">
-        <v>3382</v>
+        <v>3851</v>
       </c>
       <c r="B58" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="C58" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="D58" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="E58" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="1">
-        <v>3392</v>
+        <v>3921</v>
       </c>
       <c r="B59" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="C59" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="D59" t="s">
-        <v>57</v>
+        <v>93</v>
+      </c>
+      <c r="E59" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="1">
-        <v>3456</v>
+        <v>3991</v>
       </c>
       <c r="B60" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="C60" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D60" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E60" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="1">
-        <v>3666</v>
+        <v>4061</v>
       </c>
       <c r="B61" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="C61" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E61" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="1">
-        <v>3792</v>
+        <v>4131</v>
       </c>
       <c r="B62" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="C62" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="D62" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E62" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="1">
-        <v>3946</v>
+        <v>4201</v>
       </c>
       <c r="B63" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="C63" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="D63" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E63" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="1">
-        <v>4081</v>
+        <v>4271</v>
       </c>
       <c r="B64" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="C64" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D64" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E64" t="s">
-        <v>65</v>
+        <v>96</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="1">
-        <v>4130</v>
+        <v>4341</v>
       </c>
       <c r="B65" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="C65" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="D65" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="E65" t="s">
-        <v>56</v>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="1">
+        <v>4411</v>
+      </c>
+      <c r="B66" t="s">
+        <v>67</v>
+      </c>
+      <c r="C66" t="s">
+        <v>90</v>
+      </c>
+      <c r="D66" t="s">
+        <v>93</v>
+      </c>
+      <c r="E66" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="1">
+        <v>4481</v>
+      </c>
+      <c r="B67" t="s">
+        <v>68</v>
+      </c>
+      <c r="C67" t="s">
+        <v>90</v>
+      </c>
+      <c r="D67" t="s">
+        <v>93</v>
+      </c>
+      <c r="E67" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="1">
+        <v>4551</v>
+      </c>
+      <c r="B68" t="s">
+        <v>69</v>
+      </c>
+      <c r="C68" t="s">
+        <v>90</v>
+      </c>
+      <c r="D68" t="s">
+        <v>93</v>
+      </c>
+      <c r="E68" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="1">
+        <v>4621</v>
+      </c>
+      <c r="B69" t="s">
+        <v>70</v>
+      </c>
+      <c r="C69" t="s">
+        <v>90</v>
+      </c>
+      <c r="D69" t="s">
+        <v>93</v>
+      </c>
+      <c r="E69" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="1">
+        <v>4691</v>
+      </c>
+      <c r="B70" t="s">
+        <v>71</v>
+      </c>
+      <c r="C70" t="s">
+        <v>90</v>
+      </c>
+      <c r="D70" t="s">
+        <v>93</v>
+      </c>
+      <c r="E70" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="1">
+        <v>4761</v>
+      </c>
+      <c r="B71" t="s">
+        <v>72</v>
+      </c>
+      <c r="C71" t="s">
+        <v>90</v>
+      </c>
+      <c r="D71" t="s">
+        <v>93</v>
+      </c>
+      <c r="E71" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="1">
+        <v>4831</v>
+      </c>
+      <c r="B72" t="s">
+        <v>73</v>
+      </c>
+      <c r="C72" t="s">
+        <v>90</v>
+      </c>
+      <c r="D72" t="s">
+        <v>93</v>
+      </c>
+      <c r="E72" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="1">
+        <v>4838</v>
+      </c>
+      <c r="B73" t="s">
+        <v>73</v>
+      </c>
+      <c r="C73" t="s">
+        <v>92</v>
+      </c>
+      <c r="D73" t="s">
+        <v>94</v>
+      </c>
+      <c r="E73" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="1">
+        <v>4901</v>
+      </c>
+      <c r="B74" t="s">
+        <v>74</v>
+      </c>
+      <c r="C74" t="s">
+        <v>90</v>
+      </c>
+      <c r="D74" t="s">
+        <v>93</v>
+      </c>
+      <c r="E74" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="1">
+        <v>4971</v>
+      </c>
+      <c r="B75" t="s">
+        <v>75</v>
+      </c>
+      <c r="C75" t="s">
+        <v>90</v>
+      </c>
+      <c r="D75" t="s">
+        <v>93</v>
+      </c>
+      <c r="E75" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="1">
+        <v>5041</v>
+      </c>
+      <c r="B76" t="s">
+        <v>76</v>
+      </c>
+      <c r="C76" t="s">
+        <v>90</v>
+      </c>
+      <c r="D76" t="s">
+        <v>93</v>
+      </c>
+      <c r="E76" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="1">
+        <v>5111</v>
+      </c>
+      <c r="B77" t="s">
+        <v>77</v>
+      </c>
+      <c r="C77" t="s">
+        <v>90</v>
+      </c>
+      <c r="D77" t="s">
+        <v>93</v>
+      </c>
+      <c r="E77" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" s="1">
+        <v>5181</v>
+      </c>
+      <c r="B78" t="s">
+        <v>78</v>
+      </c>
+      <c r="C78" t="s">
+        <v>90</v>
+      </c>
+      <c r="D78" t="s">
+        <v>93</v>
+      </c>
+      <c r="E78" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" s="1">
+        <v>5251</v>
+      </c>
+      <c r="B79" t="s">
+        <v>79</v>
+      </c>
+      <c r="C79" t="s">
+        <v>90</v>
+      </c>
+      <c r="D79" t="s">
+        <v>93</v>
+      </c>
+      <c r="E79" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80" s="1">
+        <v>5321</v>
+      </c>
+      <c r="B80" t="s">
+        <v>80</v>
+      </c>
+      <c r="C80" t="s">
+        <v>90</v>
+      </c>
+      <c r="D80" t="s">
+        <v>93</v>
+      </c>
+      <c r="E80" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" s="1">
+        <v>5391</v>
+      </c>
+      <c r="B81" t="s">
+        <v>81</v>
+      </c>
+      <c r="C81" t="s">
+        <v>90</v>
+      </c>
+      <c r="D81" t="s">
+        <v>93</v>
+      </c>
+      <c r="E81" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" s="1">
+        <v>5461</v>
+      </c>
+      <c r="B82" t="s">
+        <v>82</v>
+      </c>
+      <c r="C82" t="s">
+        <v>90</v>
+      </c>
+      <c r="D82" t="s">
+        <v>93</v>
+      </c>
+      <c r="E82" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" s="1">
+        <v>5531</v>
+      </c>
+      <c r="B83" t="s">
+        <v>83</v>
+      </c>
+      <c r="C83" t="s">
+        <v>90</v>
+      </c>
+      <c r="D83" t="s">
+        <v>93</v>
+      </c>
+      <c r="E83" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" s="1">
+        <v>5601</v>
+      </c>
+      <c r="B84" t="s">
+        <v>84</v>
+      </c>
+      <c r="C84" t="s">
+        <v>90</v>
+      </c>
+      <c r="D84" t="s">
+        <v>93</v>
+      </c>
+      <c r="E84" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" s="1">
+        <v>5671</v>
+      </c>
+      <c r="B85" t="s">
+        <v>85</v>
+      </c>
+      <c r="C85" t="s">
+        <v>90</v>
+      </c>
+      <c r="D85" t="s">
+        <v>93</v>
+      </c>
+      <c r="E85" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" s="1">
+        <v>5741</v>
+      </c>
+      <c r="B86" t="s">
+        <v>86</v>
+      </c>
+      <c r="C86" t="s">
+        <v>90</v>
+      </c>
+      <c r="D86" t="s">
+        <v>93</v>
+      </c>
+      <c r="E86" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" s="1">
+        <v>5811</v>
+      </c>
+      <c r="B87" t="s">
+        <v>87</v>
+      </c>
+      <c r="C87" t="s">
+        <v>90</v>
+      </c>
+      <c r="D87" t="s">
+        <v>93</v>
+      </c>
+      <c r="E87" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88" s="1">
+        <v>5881</v>
+      </c>
+      <c r="B88" t="s">
+        <v>88</v>
+      </c>
+      <c r="C88" t="s">
+        <v>90</v>
+      </c>
+      <c r="D88" t="s">
+        <v>93</v>
+      </c>
+      <c r="E88" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89" s="1">
+        <v>5952</v>
+      </c>
+      <c r="B89" t="s">
+        <v>89</v>
+      </c>
+      <c r="C89" t="s">
+        <v>90</v>
+      </c>
+      <c r="D89" t="s">
+        <v>93</v>
+      </c>
+      <c r="E89" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
GSTP1 wordt nu uit phenotype.rpt gehaald. Genen die meerdere SNP's nodig hebben blijven nu leeg, en worden gevuld vanuit Tahar's unknowns. WIP
</commit_message>
<xml_diff>
--- a/Output/Diagnostics/unknowns.xlsx
+++ b/Output/Diagnostics/unknowns.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="98">
   <si>
     <t>sample_id</t>
   </si>
@@ -290,9 +290,6 @@
   </si>
   <si>
     <t>NQ01</t>
-  </si>
-  <si>
-    <t>BChE</t>
   </si>
   <si>
     <t>ERROR</t>
@@ -668,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -696,15 +693,15 @@
         <v>90</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -713,15 +710,15 @@
         <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
@@ -730,15 +727,15 @@
         <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1">
-        <v>211</v>
+        <v>193</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -747,15 +744,15 @@
         <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1">
-        <v>281</v>
+        <v>257</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -764,15 +761,15 @@
         <v>90</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1">
-        <v>351</v>
+        <v>321</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -781,15 +778,15 @@
         <v>90</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1">
-        <v>421</v>
+        <v>385</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
@@ -798,15 +795,15 @@
         <v>90</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1">
-        <v>491</v>
+        <v>449</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
@@ -815,15 +812,15 @@
         <v>90</v>
       </c>
       <c r="D9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1">
-        <v>561</v>
+        <v>513</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
@@ -832,15 +829,15 @@
         <v>90</v>
       </c>
       <c r="D10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1">
-        <v>631</v>
+        <v>577</v>
       </c>
       <c r="B11" t="s">
         <v>13</v>
@@ -849,15 +846,15 @@
         <v>90</v>
       </c>
       <c r="D11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1">
-        <v>701</v>
+        <v>641</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
@@ -866,15 +863,15 @@
         <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1">
-        <v>771</v>
+        <v>705</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
@@ -883,15 +880,15 @@
         <v>90</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1">
-        <v>841</v>
+        <v>769</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
@@ -900,15 +897,15 @@
         <v>90</v>
       </c>
       <c r="D14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1">
-        <v>911</v>
+        <v>833</v>
       </c>
       <c r="B15" t="s">
         <v>17</v>
@@ -917,15 +914,15 @@
         <v>90</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1">
-        <v>981</v>
+        <v>897</v>
       </c>
       <c r="B16" t="s">
         <v>18</v>
@@ -934,15 +931,15 @@
         <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1">
-        <v>1051</v>
+        <v>961</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
@@ -951,15 +948,15 @@
         <v>90</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1">
-        <v>1121</v>
+        <v>1025</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
@@ -968,15 +965,15 @@
         <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1">
-        <v>1191</v>
+        <v>1089</v>
       </c>
       <c r="B19" t="s">
         <v>21</v>
@@ -985,15 +982,15 @@
         <v>90</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1">
-        <v>1261</v>
+        <v>1153</v>
       </c>
       <c r="B20" t="s">
         <v>22</v>
@@ -1002,15 +999,15 @@
         <v>90</v>
       </c>
       <c r="D20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1">
-        <v>1331</v>
+        <v>1217</v>
       </c>
       <c r="B21" t="s">
         <v>23</v>
@@ -1019,15 +1016,15 @@
         <v>90</v>
       </c>
       <c r="D21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1">
-        <v>1401</v>
+        <v>1281</v>
       </c>
       <c r="B22" t="s">
         <v>24</v>
@@ -1036,15 +1033,15 @@
         <v>90</v>
       </c>
       <c r="D22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1">
-        <v>1471</v>
+        <v>1345</v>
       </c>
       <c r="B23" t="s">
         <v>25</v>
@@ -1053,15 +1050,15 @@
         <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E23" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1">
-        <v>1541</v>
+        <v>1409</v>
       </c>
       <c r="B24" t="s">
         <v>26</v>
@@ -1070,15 +1067,15 @@
         <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E24" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1">
-        <v>1611</v>
+        <v>1473</v>
       </c>
       <c r="B25" t="s">
         <v>27</v>
@@ -1087,15 +1084,15 @@
         <v>90</v>
       </c>
       <c r="D25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1">
-        <v>1681</v>
+        <v>1537</v>
       </c>
       <c r="B26" t="s">
         <v>28</v>
@@ -1104,15 +1101,15 @@
         <v>90</v>
       </c>
       <c r="D26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E26" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1">
-        <v>1751</v>
+        <v>1601</v>
       </c>
       <c r="B27" t="s">
         <v>29</v>
@@ -1121,15 +1118,15 @@
         <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E27" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1">
-        <v>1821</v>
+        <v>1665</v>
       </c>
       <c r="B28" t="s">
         <v>30</v>
@@ -1138,15 +1135,15 @@
         <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E28" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1">
-        <v>1891</v>
+        <v>1729</v>
       </c>
       <c r="B29" t="s">
         <v>31</v>
@@ -1155,15 +1152,15 @@
         <v>90</v>
       </c>
       <c r="D29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E29" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1">
-        <v>1961</v>
+        <v>1793</v>
       </c>
       <c r="B30" t="s">
         <v>32</v>
@@ -1172,15 +1169,15 @@
         <v>90</v>
       </c>
       <c r="D30" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E30" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1">
-        <v>2031</v>
+        <v>1857</v>
       </c>
       <c r="B31" t="s">
         <v>33</v>
@@ -1189,15 +1186,15 @@
         <v>90</v>
       </c>
       <c r="D31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1">
-        <v>2101</v>
+        <v>1921</v>
       </c>
       <c r="B32" t="s">
         <v>34</v>
@@ -1206,15 +1203,15 @@
         <v>90</v>
       </c>
       <c r="D32" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="1">
-        <v>2171</v>
+        <v>1985</v>
       </c>
       <c r="B33" t="s">
         <v>35</v>
@@ -1223,15 +1220,15 @@
         <v>90</v>
       </c>
       <c r="D33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E33" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="1">
-        <v>2241</v>
+        <v>2049</v>
       </c>
       <c r="B34" t="s">
         <v>36</v>
@@ -1240,15 +1237,15 @@
         <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="1">
-        <v>2311</v>
+        <v>2113</v>
       </c>
       <c r="B35" t="s">
         <v>37</v>
@@ -1257,15 +1254,15 @@
         <v>90</v>
       </c>
       <c r="D35" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="1">
-        <v>2381</v>
+        <v>2177</v>
       </c>
       <c r="B36" t="s">
         <v>38</v>
@@ -1274,15 +1271,15 @@
         <v>90</v>
       </c>
       <c r="D36" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="1">
-        <v>2451</v>
+        <v>2241</v>
       </c>
       <c r="B37" t="s">
         <v>39</v>
@@ -1291,15 +1288,15 @@
         <v>90</v>
       </c>
       <c r="D37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E37" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="1">
-        <v>2521</v>
+        <v>2305</v>
       </c>
       <c r="B38" t="s">
         <v>40</v>
@@ -1308,15 +1305,15 @@
         <v>90</v>
       </c>
       <c r="D38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1">
-        <v>2591</v>
+        <v>2369</v>
       </c>
       <c r="B39" t="s">
         <v>41</v>
@@ -1325,15 +1322,15 @@
         <v>90</v>
       </c>
       <c r="D39" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E39" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="1">
-        <v>2661</v>
+        <v>2433</v>
       </c>
       <c r="B40" t="s">
         <v>42</v>
@@ -1342,15 +1339,15 @@
         <v>90</v>
       </c>
       <c r="D40" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E40" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1">
-        <v>2731</v>
+        <v>2497</v>
       </c>
       <c r="B41" t="s">
         <v>43</v>
@@ -1359,15 +1356,15 @@
         <v>90</v>
       </c>
       <c r="D41" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E41" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="1">
-        <v>2801</v>
+        <v>2561</v>
       </c>
       <c r="B42" t="s">
         <v>44</v>
@@ -1376,15 +1373,15 @@
         <v>90</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E42" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="1">
-        <v>2871</v>
+        <v>2625</v>
       </c>
       <c r="B43" t="s">
         <v>45</v>
@@ -1393,15 +1390,15 @@
         <v>90</v>
       </c>
       <c r="D43" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E43" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="1">
-        <v>2941</v>
+        <v>2689</v>
       </c>
       <c r="B44" t="s">
         <v>46</v>
@@ -1410,15 +1407,15 @@
         <v>90</v>
       </c>
       <c r="D44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E44" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="1">
-        <v>3011</v>
+        <v>2753</v>
       </c>
       <c r="B45" t="s">
         <v>47</v>
@@ -1427,15 +1424,15 @@
         <v>90</v>
       </c>
       <c r="D45" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E45" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="1">
-        <v>3081</v>
+        <v>2817</v>
       </c>
       <c r="B46" t="s">
         <v>48</v>
@@ -1444,15 +1441,15 @@
         <v>90</v>
       </c>
       <c r="D46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E46" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="1">
-        <v>3151</v>
+        <v>2881</v>
       </c>
       <c r="B47" t="s">
         <v>49</v>
@@ -1461,15 +1458,15 @@
         <v>90</v>
       </c>
       <c r="D47" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E47" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="1">
-        <v>3221</v>
+        <v>2945</v>
       </c>
       <c r="B48" t="s">
         <v>50</v>
@@ -1478,15 +1475,15 @@
         <v>90</v>
       </c>
       <c r="D48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="1">
-        <v>3291</v>
+        <v>3009</v>
       </c>
       <c r="B49" t="s">
         <v>51</v>
@@ -1495,15 +1492,15 @@
         <v>90</v>
       </c>
       <c r="D49" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E49" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="1">
-        <v>3361</v>
+        <v>3073</v>
       </c>
       <c r="B50" t="s">
         <v>52</v>
@@ -1512,15 +1509,15 @@
         <v>90</v>
       </c>
       <c r="D50" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E50" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="1">
-        <v>3431</v>
+        <v>3137</v>
       </c>
       <c r="B51" t="s">
         <v>53</v>
@@ -1529,15 +1526,15 @@
         <v>90</v>
       </c>
       <c r="D51" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E51" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="1">
-        <v>3501</v>
+        <v>3201</v>
       </c>
       <c r="B52" t="s">
         <v>54</v>
@@ -1546,15 +1543,15 @@
         <v>90</v>
       </c>
       <c r="D52" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E52" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="1">
-        <v>3571</v>
+        <v>3265</v>
       </c>
       <c r="B53" t="s">
         <v>55</v>
@@ -1563,15 +1560,15 @@
         <v>90</v>
       </c>
       <c r="D53" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E53" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="1">
-        <v>3641</v>
+        <v>3329</v>
       </c>
       <c r="B54" t="s">
         <v>56</v>
@@ -1580,15 +1577,15 @@
         <v>90</v>
       </c>
       <c r="D54" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E54" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="1">
-        <v>3711</v>
+        <v>3393</v>
       </c>
       <c r="B55" t="s">
         <v>57</v>
@@ -1597,15 +1594,15 @@
         <v>90</v>
       </c>
       <c r="D55" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E55" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="1">
-        <v>3764</v>
+        <v>3441</v>
       </c>
       <c r="B56" t="s">
         <v>57</v>
@@ -1614,15 +1611,15 @@
         <v>91</v>
       </c>
       <c r="D56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E56" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="1">
-        <v>3781</v>
+        <v>3457</v>
       </c>
       <c r="B57" t="s">
         <v>58</v>
@@ -1631,15 +1628,15 @@
         <v>90</v>
       </c>
       <c r="D57" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E57" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="1">
-        <v>3851</v>
+        <v>3521</v>
       </c>
       <c r="B58" t="s">
         <v>59</v>
@@ -1648,15 +1645,15 @@
         <v>90</v>
       </c>
       <c r="D58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E58" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="1">
-        <v>3921</v>
+        <v>3585</v>
       </c>
       <c r="B59" t="s">
         <v>60</v>
@@ -1665,15 +1662,15 @@
         <v>90</v>
       </c>
       <c r="D59" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E59" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="1">
-        <v>3991</v>
+        <v>3649</v>
       </c>
       <c r="B60" t="s">
         <v>61</v>
@@ -1682,15 +1679,15 @@
         <v>90</v>
       </c>
       <c r="D60" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E60" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="1">
-        <v>4061</v>
+        <v>3713</v>
       </c>
       <c r="B61" t="s">
         <v>62</v>
@@ -1699,15 +1696,15 @@
         <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E61" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="1">
-        <v>4131</v>
+        <v>3777</v>
       </c>
       <c r="B62" t="s">
         <v>63</v>
@@ -1716,15 +1713,15 @@
         <v>90</v>
       </c>
       <c r="D62" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E62" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="1">
-        <v>4201</v>
+        <v>3841</v>
       </c>
       <c r="B63" t="s">
         <v>64</v>
@@ -1733,15 +1730,15 @@
         <v>90</v>
       </c>
       <c r="D63" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E63" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="1">
-        <v>4271</v>
+        <v>3905</v>
       </c>
       <c r="B64" t="s">
         <v>65</v>
@@ -1750,15 +1747,15 @@
         <v>90</v>
       </c>
       <c r="D64" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E64" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="1">
-        <v>4341</v>
+        <v>3969</v>
       </c>
       <c r="B65" t="s">
         <v>66</v>
@@ -1767,15 +1764,15 @@
         <v>90</v>
       </c>
       <c r="D65" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E65" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="1">
-        <v>4411</v>
+        <v>4033</v>
       </c>
       <c r="B66" t="s">
         <v>67</v>
@@ -1784,15 +1781,15 @@
         <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E66" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="1">
-        <v>4481</v>
+        <v>4097</v>
       </c>
       <c r="B67" t="s">
         <v>68</v>
@@ -1801,15 +1798,15 @@
         <v>90</v>
       </c>
       <c r="D67" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E67" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="1">
-        <v>4551</v>
+        <v>4161</v>
       </c>
       <c r="B68" t="s">
         <v>69</v>
@@ -1818,15 +1815,15 @@
         <v>90</v>
       </c>
       <c r="D68" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E68" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="1">
-        <v>4621</v>
+        <v>4225</v>
       </c>
       <c r="B69" t="s">
         <v>70</v>
@@ -1835,15 +1832,15 @@
         <v>90</v>
       </c>
       <c r="D69" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E69" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" s="1">
-        <v>4691</v>
+        <v>4289</v>
       </c>
       <c r="B70" t="s">
         <v>71</v>
@@ -1852,15 +1849,15 @@
         <v>90</v>
       </c>
       <c r="D70" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E70" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="1">
-        <v>4761</v>
+        <v>4353</v>
       </c>
       <c r="B71" t="s">
         <v>72</v>
@@ -1869,15 +1866,15 @@
         <v>90</v>
       </c>
       <c r="D71" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E71" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="1">
-        <v>4831</v>
+        <v>4417</v>
       </c>
       <c r="B72" t="s">
         <v>73</v>
@@ -1886,75 +1883,75 @@
         <v>90</v>
       </c>
       <c r="D72" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E72" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" s="1">
-        <v>4838</v>
+        <v>4481</v>
       </c>
       <c r="B73" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C73" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D73" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E73" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" s="1">
-        <v>4901</v>
+        <v>4545</v>
       </c>
       <c r="B74" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C74" t="s">
         <v>90</v>
       </c>
       <c r="D74" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E74" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="1">
-        <v>4971</v>
+        <v>4609</v>
       </c>
       <c r="B75" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C75" t="s">
         <v>90</v>
       </c>
       <c r="D75" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E75" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" s="1">
-        <v>5041</v>
+        <v>4673</v>
       </c>
       <c r="B76" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C76" t="s">
         <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E76" t="s">
         <v>95</v>
@@ -1962,152 +1959,152 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" s="1">
-        <v>5111</v>
+        <v>4737</v>
       </c>
       <c r="B77" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C77" t="s">
         <v>90</v>
       </c>
       <c r="D77" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E77" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" s="1">
-        <v>5181</v>
+        <v>4801</v>
       </c>
       <c r="B78" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C78" t="s">
         <v>90</v>
       </c>
       <c r="D78" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E78" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" s="1">
-        <v>5251</v>
+        <v>4865</v>
       </c>
       <c r="B79" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C79" t="s">
         <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E79" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" s="1">
-        <v>5321</v>
+        <v>4929</v>
       </c>
       <c r="B80" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C80" t="s">
         <v>90</v>
       </c>
       <c r="D80" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E80" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" s="1">
-        <v>5391</v>
+        <v>4993</v>
       </c>
       <c r="B81" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C81" t="s">
         <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E81" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" s="1">
-        <v>5461</v>
+        <v>5057</v>
       </c>
       <c r="B82" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C82" t="s">
         <v>90</v>
       </c>
       <c r="D82" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E82" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" s="1">
-        <v>5531</v>
+        <v>5121</v>
       </c>
       <c r="B83" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C83" t="s">
         <v>90</v>
       </c>
       <c r="D83" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E83" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84" s="1">
-        <v>5601</v>
+        <v>5185</v>
       </c>
       <c r="B84" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C84" t="s">
         <v>90</v>
       </c>
       <c r="D84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E84" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="85" spans="1:5">
       <c r="A85" s="1">
-        <v>5671</v>
+        <v>5249</v>
       </c>
       <c r="B85" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C85" t="s">
         <v>90</v>
       </c>
       <c r="D85" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E85" t="s">
         <v>95</v>
@@ -2115,70 +2112,53 @@
     </row>
     <row r="86" spans="1:5">
       <c r="A86" s="1">
-        <v>5741</v>
+        <v>5313</v>
       </c>
       <c r="B86" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C86" t="s">
         <v>90</v>
       </c>
       <c r="D86" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E86" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="87" spans="1:5">
       <c r="A87" s="1">
-        <v>5811</v>
+        <v>5377</v>
       </c>
       <c r="B87" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C87" t="s">
         <v>90</v>
       </c>
       <c r="D87" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E87" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" s="1">
-        <v>5881</v>
+        <v>5442</v>
       </c>
       <c r="B88" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C88" t="s">
         <v>90</v>
       </c>
       <c r="D88" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E88" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5">
-      <c r="A89" s="1">
-        <v>5952</v>
-      </c>
-      <c r="B89" t="s">
-        <v>89</v>
-      </c>
-      <c r="C89" t="s">
-        <v>90</v>
-      </c>
-      <c r="D89" t="s">
-        <v>93</v>
-      </c>
-      <c r="E89" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>